<commit_message>
refactor(certificados): renombrar _procesarCertificadoTributario a _procesarCertificadoAEAT
Se renombra la función para usar una denominación más clara y consistente con el
acrónimo de la Agencia Estatal de Administración Tributaria (AEAT).

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/procesos/inputs/Excel CCC Empresas.xlsx
+++ b/procesos/inputs/Excel CCC Empresas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\OneDrive\Nodus\Proyectos\Nodus-app\parche-gestoria\procesos\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72DBD40A-3B58-4993-AA95-C70F225C335A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{320CCD95-5745-4A57-8267-90C79DE2569C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14595" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,9 +16,9 @@
     <sheet name="BASE DE DATOS (NO TOCAR)" sheetId="14" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BASE DE DATOS (NO TOCAR)'!$A$1:$K$254</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BASE DE DATOS (NO TOCAR)'!$A$1:$J$254</definedName>
   </definedNames>
-  <calcPr calcId="191029"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1289" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="826">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -2617,7 +2617,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
@@ -2658,6 +2658,9 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -3069,13 +3072,13 @@
         <v>823</v>
       </c>
       <c r="I1" s="9" t="s">
+        <v>821</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>822</v>
+      </c>
+      <c r="K1" s="9" t="s">
         <v>824</v>
-      </c>
-      <c r="J1" s="9" t="s">
-        <v>821</v>
-      </c>
-      <c r="K1" s="9" t="s">
-        <v>822</v>
       </c>
     </row>
     <row r="2" spans="1:11" x14ac:dyDescent="0.35">
@@ -3185,10 +3188,10 @@
       <c r="G5" s="16" t="s">
         <v>383</v>
       </c>
-      <c r="H5" s="19"/>
-      <c r="I5" s="19"/>
+      <c r="H5" s="22"/>
+      <c r="I5" s="22"/>
       <c r="J5" s="19"/>
-      <c r="K5" s="19"/>
+      <c r="K5" s="22"/>
     </row>
     <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
@@ -3245,10 +3248,10 @@
         <v>825</v>
       </c>
       <c r="I7" s="19"/>
-      <c r="J7" s="19"/>
-      <c r="K7" s="19" t="s">
+      <c r="J7" s="19" t="s">
         <v>825</v>
       </c>
+      <c r="K7" s="19"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
@@ -3276,9 +3279,7 @@
       <c r="H8" s="19"/>
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
-      <c r="K8" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="K8" s="19"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
@@ -3304,9 +3305,7 @@
         <v>389</v>
       </c>
       <c r="H9" s="19"/>
-      <c r="I9" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="I9" s="19"/>
       <c r="J9" s="19"/>
       <c r="K9" s="19"/>
     </row>
@@ -3333,10 +3332,10 @@
       <c r="G10" s="16" t="s">
         <v>389</v>
       </c>
-      <c r="H10" s="19"/>
-      <c r="I10" s="19"/>
+      <c r="H10" s="22"/>
+      <c r="I10" s="22"/>
       <c r="J10" s="19"/>
-      <c r="K10" s="19"/>
+      <c r="K10" s="22"/>
     </row>
     <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
@@ -3389,10 +3388,18 @@
       <c r="G12" s="16" t="s">
         <v>393</v>
       </c>
-      <c r="H12" s="19"/>
-      <c r="I12" s="19"/>
-      <c r="J12" s="19"/>
-      <c r="K12" s="19"/>
+      <c r="H12" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="I12" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="J12" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="K12" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
@@ -3417,15 +3424,9 @@
       <c r="G13" s="16" t="s">
         <v>382</v>
       </c>
-      <c r="H13" s="19" t="s">
-        <v>825</v>
-      </c>
-      <c r="I13" s="19" t="s">
-        <v>825</v>
-      </c>
-      <c r="J13" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="H13" s="19"/>
+      <c r="I13" s="19"/>
+      <c r="J13" s="19"/>
       <c r="K13" s="19"/>
     </row>
     <row r="14" spans="1:11" x14ac:dyDescent="0.35">
@@ -3451,15 +3452,9 @@
       <c r="G14" s="16" t="s">
         <v>382</v>
       </c>
-      <c r="H14" s="19" t="s">
-        <v>825</v>
-      </c>
-      <c r="I14" s="19" t="s">
-        <v>825</v>
-      </c>
-      <c r="J14" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="H14" s="19"/>
+      <c r="I14" s="19"/>
+      <c r="J14" s="19"/>
       <c r="K14" s="19"/>
     </row>
     <row r="15" spans="1:11" x14ac:dyDescent="0.35">
@@ -3488,9 +3483,7 @@
       <c r="H15" s="19"/>
       <c r="I15" s="19"/>
       <c r="J15" s="19"/>
-      <c r="K15" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="K15" s="19"/>
     </row>
     <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
@@ -3517,9 +3510,7 @@
       </c>
       <c r="H16" s="19"/>
       <c r="I16" s="19"/>
-      <c r="J16" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="J16" s="19"/>
       <c r="K16" s="19"/>
     </row>
     <row r="17" spans="1:11" x14ac:dyDescent="0.35">

</xml_diff>

<commit_message>
feat: eliminar dependencia en config.json para certificados AEAT
- Remover archivo config.json (ya no necesario)
- Sistema ahora busca certificados automáticamente por NIF desde almacén Windows
- Soporta certificados directos (personas) y representantes (empresas)
- Excel CCC Empresas.xlsx es la única fuente de verdad

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/procesos/inputs/Excel CCC Empresas.xlsx
+++ b/procesos/inputs/Excel CCC Empresas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\OneDrive\Nodus\Proyectos\Nodus-app\parche-gestoria\procesos\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{320CCD95-5745-4A57-8267-90C79DE2569C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD454C1B-0158-4083-9BF7-A71E771EED16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14595" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="BASE DE DATOS (NO TOCAR)" sheetId="14" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BASE DE DATOS (NO TOCAR)'!$A$1:$J$254</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'BASE DE DATOS (NO TOCAR)'!$A$1:$K$254</definedName>
   </definedNames>
   <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1283" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1296" uniqueCount="826">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -3244,13 +3244,9 @@
       <c r="G7" s="16" t="s">
         <v>385</v>
       </c>
-      <c r="H7" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="H7" s="19"/>
       <c r="I7" s="19"/>
-      <c r="J7" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="J7" s="19"/>
       <c r="K7" s="19"/>
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.35">
@@ -3279,7 +3275,9 @@
       <c r="H8" s="19"/>
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
-      <c r="K8" s="19"/>
+      <c r="K8" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
@@ -4460,10 +4458,18 @@
       <c r="G50" s="16" t="s">
         <v>454</v>
       </c>
-      <c r="H50" s="19"/>
-      <c r="I50" s="19"/>
-      <c r="J50" s="19"/>
-      <c r="K50" s="19"/>
+      <c r="H50" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="I50" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="J50" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="K50" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
@@ -4488,10 +4494,18 @@
       <c r="G51" s="16" t="s">
         <v>454</v>
       </c>
-      <c r="H51" s="19"/>
-      <c r="I51" s="19"/>
-      <c r="J51" s="19"/>
-      <c r="K51" s="19"/>
+      <c r="H51" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="I51" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="J51" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="K51" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
@@ -7316,10 +7330,16 @@
       <c r="G152" s="16" t="s">
         <v>387</v>
       </c>
-      <c r="H152" s="19"/>
-      <c r="I152" s="19"/>
+      <c r="H152" s="19" t="s">
+        <v>825</v>
+      </c>
+      <c r="I152" s="19" t="s">
+        <v>825</v>
+      </c>
       <c r="J152" s="19"/>
-      <c r="K152" s="19"/>
+      <c r="K152" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
@@ -7627,7 +7647,9 @@
       <c r="H163" s="19"/>
       <c r="I163" s="19"/>
       <c r="J163" s="19"/>
-      <c r="K163" s="19"/>
+      <c r="K163" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="164" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
@@ -8355,7 +8377,9 @@
       <c r="H189" s="19"/>
       <c r="I189" s="19"/>
       <c r="J189" s="19"/>
-      <c r="K189" s="19"/>
+      <c r="K189" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="190" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
@@ -8719,7 +8743,9 @@
       <c r="H202" s="19"/>
       <c r="I202" s="19"/>
       <c r="J202" s="19"/>
-      <c r="K202" s="19"/>
+      <c r="K202" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="203" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
@@ -10177,6 +10203,7 @@
       <c r="K254" s="19"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:K254" xr:uid="{00000000-0001-0000-0100-000000000000}"/>
   <hyperlinks>
     <hyperlink ref="G254" r:id="rId1" xr:uid="{99771A5B-A528-4903-9C40-A57E66882FE1}"/>
   </hyperlinks>
@@ -10195,12 +10222,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AF0C36E9CBDE43468AAB846756A8BA94" ma:contentTypeVersion="0" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="93c275e25462616b2c1de9b58ec156dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f6edc329ff236629c56e3b879b320d0">
     <xsd:element name="properties">
@@ -10314,6 +10335,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DDD49F8-6691-4324-BC0D-0B1E4890A2C6}">
   <ds:schemaRefs>
@@ -10323,21 +10350,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEFD23-736F-4CE9-81DA-D9D145B9B572}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A01C7383-C303-4DC2-9970-99C89A193825}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10351,4 +10363,19 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEFD23-736F-4CE9-81DA-D9D145B9B572}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(certificados): seleccionar 'En nombre propio' en formulario AEAT
Corrige el ID del radio button para seleccionar "En nombre propio" (fTipoRepresentacion0) en lugar de "En representación de terceros" (fTipoRepresentacion1).

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/procesos/inputs/Excel CCC Empresas.xlsx
+++ b/procesos/inputs/Excel CCC Empresas.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\OneDrive\Nodus\Proyectos\Nodus-app\parche-gestoria\procesos\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AD454C1B-0158-4083-9BF7-A71E771EED16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D8B8180-7D09-47FF-9444-9131E349C0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-14595" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE DE DATOS (NO TOCAR)" sheetId="14" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1296" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1294" uniqueCount="826">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -3275,9 +3275,7 @@
       <c r="H8" s="19"/>
       <c r="I8" s="19"/>
       <c r="J8" s="19"/>
-      <c r="K8" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="K8" s="19"/>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
@@ -7337,9 +7335,7 @@
         <v>825</v>
       </c>
       <c r="J152" s="19"/>
-      <c r="K152" s="19" t="s">
-        <v>825</v>
-      </c>
+      <c r="K152" s="19"/>
     </row>
     <row r="153" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
@@ -10222,6 +10218,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AF0C36E9CBDE43468AAB846756A8BA94" ma:contentTypeVersion="0" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="93c275e25462616b2c1de9b58ec156dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f6edc329ff236629c56e3b879b320d0">
     <xsd:element name="properties">
@@ -10335,12 +10337,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DDD49F8-6691-4324-BC0D-0B1E4890A2C6}">
   <ds:schemaRefs>
@@ -10350,6 +10346,21 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEFD23-736F-4CE9-81DA-D9D145B9B572}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A01C7383-C303-4DC2-9970-99C89A193825}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10363,19 +10374,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEFD23-736F-4CE9-81DA-D9D145B9B572}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(certificados): elevar UAC una sola vez al inicio para permisos de registro en AEAT
En equipos con la rama HKCU\Software\Policies restringida, la escritura
en el registro fallaba con acceso denegado en cada cliente, provocando un
diálogo UAC por empresa procesada.

Se añade _garantizarPermisoRegistroCerts(), invocada una única vez en la
pre-inicialización TRIB, que detecta si el usuario puede escribir en la
clave y, si no, eleva una sola vez para crear la clave y conceder
FullControl permanente. Se corrige además _setAutoSelectPolicy para
omitir New-Item cuando la clave ya existe, evitando el acceso denegado
en ejecuciones posteriores.
</commit_message>
<xml_diff>
--- a/procesos/inputs/Excel CCC Empresas.xlsx
+++ b/procesos/inputs/Excel CCC Empresas.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\OneDrive\Nodus\Proyectos\Nodus-app\parche-gestoria\procesos\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEECCF61-CF74-4EC7-BC91-C9DB9055BA29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8DA043-1D93-4251-915B-6B03C80601E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-14595" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1298" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="826">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -3309,7 +3309,9 @@
       <c r="J8" s="19" t="s">
         <v>825</v>
       </c>
-      <c r="K8" s="19"/>
+      <c r="K8" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
@@ -6615,7 +6617,9 @@
       <c r="H126" s="19"/>
       <c r="I126" s="19"/>
       <c r="J126" s="19"/>
-      <c r="K126" s="19"/>
+      <c r="K126" s="19" t="s">
+        <v>825</v>
+      </c>
     </row>
     <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
@@ -10226,6 +10230,12 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AF0C36E9CBDE43468AAB846756A8BA94" ma:contentTypeVersion="0" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="93c275e25462616b2c1de9b58ec156dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f6edc329ff236629c56e3b879b320d0">
     <xsd:element name="properties">
@@ -10339,12 +10349,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DDD49F8-6691-4324-BC0D-0B1E4890A2C6}">
   <ds:schemaRefs>
@@ -10354,6 +10358,21 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEFD23-736F-4CE9-81DA-D9D145B9B572}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A01C7383-C303-4DC2-9970-99C89A193825}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10367,19 +10386,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEFD23-736F-4CE9-81DA-D9D145B9B572}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(certificados): renombrar nombre de archivo ITA de CERT CORRIENTE a Informe ITA
</commit_message>
<xml_diff>
--- a/procesos/inputs/Excel CCC Empresas.xlsx
+++ b/procesos/inputs/Excel CCC Empresas.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="25601"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\preprod\Documents\Proyectos\parche-gestoria\procesos\inputs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\gonza\OneDrive\Nodus\Proyectos\Nodus-app\parche-gestoria\procesos\inputs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A46477AE-7687-4240-9241-1A2B24D5572D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E8DA043-1D93-4251-915B-6B03C80601E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-14595" yWindow="-16350" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BASE DE DATOS (NO TOCAR)" sheetId="14" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1301" uniqueCount="826">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1300" uniqueCount="826">
   <si>
     <t>EMPRESA</t>
   </si>
@@ -3033,20 +3033,20 @@
     <tabColor rgb="FFFFC000"/>
   </sheetPr>
   <dimension ref="A1:K254"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="10.5703125" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="42.42578125" style="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="12" customWidth="1"/>
-    <col min="4" max="4" width="14.140625" style="8" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="27.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="10.85546875" style="6" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="58.7109375" style="6" customWidth="1"/>
-    <col min="8" max="11" width="10.85546875" style="21"/>
-    <col min="12" max="16384" width="10.85546875" style="6"/>
+    <col min="1" max="1" width="10.54296875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="42.453125" style="6" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.1796875" style="12" customWidth="1"/>
+    <col min="4" max="4" width="14.1796875" style="8" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="27.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="10.81640625" style="6" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="58.7265625" style="6" customWidth="1"/>
+    <col min="8" max="11" width="10.81640625" style="21"/>
+    <col min="12" max="16384" width="10.81640625" style="6"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" s="9" t="s">
         <v>815</v>
       </c>
@@ -3081,7 +3081,7 @@
         <v>824</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2" s="2" t="s">
         <v>40</v>
       </c>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="K2" s="19"/>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A3" s="2" t="s">
         <v>40</v>
       </c>
@@ -3149,7 +3149,7 @@
       </c>
       <c r="K3" s="19"/>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A4" s="2" t="s">
         <v>40</v>
       </c>
@@ -3183,7 +3183,7 @@
       </c>
       <c r="K4" s="19"/>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A5" s="2" t="s">
         <v>40</v>
       </c>
@@ -3217,7 +3217,7 @@
       </c>
       <c r="K5" s="22"/>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A6" s="2" t="s">
         <v>40</v>
       </c>
@@ -3251,7 +3251,7 @@
       </c>
       <c r="K6" s="19"/>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A7" s="2" t="s">
         <v>41</v>
       </c>
@@ -3279,7 +3279,7 @@
       <c r="J7" s="19"/>
       <c r="K7" s="19"/>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A8" s="2" t="s">
         <v>215</v>
       </c>
@@ -3309,9 +3309,11 @@
       <c r="J8" s="19" t="s">
         <v>825</v>
       </c>
-      <c r="K8" s="19"/>
-    </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K8" s="19" t="s">
+        <v>825</v>
+      </c>
+    </row>
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A9" s="2" t="s">
         <v>43</v>
       </c>
@@ -3339,7 +3341,7 @@
       <c r="J9" s="19"/>
       <c r="K9" s="19"/>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A10" s="2" t="s">
         <v>43</v>
       </c>
@@ -3367,7 +3369,7 @@
       <c r="J10" s="19"/>
       <c r="K10" s="22"/>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11" s="2" t="s">
         <v>45</v>
       </c>
@@ -3397,7 +3399,7 @@
       <c r="J11" s="19"/>
       <c r="K11" s="19"/>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12" s="2" t="s">
         <v>47</v>
       </c>
@@ -3425,7 +3427,7 @@
       <c r="J12" s="19"/>
       <c r="K12" s="19"/>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13" s="2" t="s">
         <v>49</v>
       </c>
@@ -3453,7 +3455,7 @@
       <c r="J13" s="19"/>
       <c r="K13" s="19"/>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14" s="2" t="s">
         <v>49</v>
       </c>
@@ -3481,7 +3483,7 @@
       <c r="J14" s="19"/>
       <c r="K14" s="19"/>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15" s="2" t="s">
         <v>50</v>
       </c>
@@ -3509,7 +3511,7 @@
       <c r="J15" s="19"/>
       <c r="K15" s="19"/>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16" s="2" t="s">
         <v>50</v>
       </c>
@@ -3537,7 +3539,7 @@
       <c r="J16" s="19"/>
       <c r="K16" s="19"/>
     </row>
-    <row r="17" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A17" s="2" t="s">
         <v>223</v>
       </c>
@@ -3565,7 +3567,7 @@
       <c r="J17" s="19"/>
       <c r="K17" s="19"/>
     </row>
-    <row r="18" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A18" s="2" t="s">
         <v>223</v>
       </c>
@@ -3593,7 +3595,7 @@
       <c r="J18" s="19"/>
       <c r="K18" s="19"/>
     </row>
-    <row r="19" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A19" s="2" t="s">
         <v>223</v>
       </c>
@@ -3621,7 +3623,7 @@
       <c r="J19" s="19"/>
       <c r="K19" s="19"/>
     </row>
-    <row r="20" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A20" s="2" t="s">
         <v>51</v>
       </c>
@@ -3649,7 +3651,7 @@
       <c r="J20" s="19"/>
       <c r="K20" s="19"/>
     </row>
-    <row r="21" spans="1:11" ht="12.75" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:11" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>112</v>
       </c>
@@ -3677,7 +3679,7 @@
       <c r="J21" s="19"/>
       <c r="K21" s="19"/>
     </row>
-    <row r="22" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A22" s="2" t="s">
         <v>52</v>
       </c>
@@ -3705,7 +3707,7 @@
       <c r="J22" s="19"/>
       <c r="K22" s="19"/>
     </row>
-    <row r="23" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A23" s="2" t="s">
         <v>52</v>
       </c>
@@ -3733,7 +3735,7 @@
       <c r="J23" s="19"/>
       <c r="K23" s="19"/>
     </row>
-    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A24" s="2" t="s">
         <v>236</v>
       </c>
@@ -3761,7 +3763,7 @@
       <c r="J24" s="19"/>
       <c r="K24" s="19"/>
     </row>
-    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A25" s="2" t="s">
         <v>54</v>
       </c>
@@ -3789,7 +3791,7 @@
       <c r="J25" s="19"/>
       <c r="K25" s="19"/>
     </row>
-    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A26" s="2" t="s">
         <v>55</v>
       </c>
@@ -3817,7 +3819,7 @@
       <c r="J26" s="19"/>
       <c r="K26" s="19"/>
     </row>
-    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A27" s="2" t="s">
         <v>57</v>
       </c>
@@ -3845,7 +3847,7 @@
       <c r="J27" s="19"/>
       <c r="K27" s="19"/>
     </row>
-    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A28" s="2" t="s">
         <v>59</v>
       </c>
@@ -3873,7 +3875,7 @@
       <c r="J28" s="19"/>
       <c r="K28" s="19"/>
     </row>
-    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A29" s="2" t="s">
         <v>61</v>
       </c>
@@ -3901,7 +3903,7 @@
       <c r="J29" s="19"/>
       <c r="K29" s="19"/>
     </row>
-    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A30" s="2" t="s">
         <v>61</v>
       </c>
@@ -3929,7 +3931,7 @@
       <c r="J30" s="19"/>
       <c r="K30" s="19"/>
     </row>
-    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A31" s="2" t="s">
         <v>62</v>
       </c>
@@ -3957,7 +3959,7 @@
       <c r="J31" s="19"/>
       <c r="K31" s="19"/>
     </row>
-    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A32" s="2" t="s">
         <v>63</v>
       </c>
@@ -3985,7 +3987,7 @@
       <c r="J32" s="19"/>
       <c r="K32" s="19"/>
     </row>
-    <row r="33" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A33" s="2" t="s">
         <v>208</v>
       </c>
@@ -4013,7 +4015,7 @@
       <c r="J33" s="19"/>
       <c r="K33" s="19"/>
     </row>
-    <row r="34" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A34" s="2" t="s">
         <v>65</v>
       </c>
@@ -4041,7 +4043,7 @@
       <c r="J34" s="19"/>
       <c r="K34" s="19"/>
     </row>
-    <row r="35" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A35" s="2" t="s">
         <v>238</v>
       </c>
@@ -4069,7 +4071,7 @@
       <c r="J35" s="19"/>
       <c r="K35" s="19"/>
     </row>
-    <row r="36" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A36" s="2" t="s">
         <v>113</v>
       </c>
@@ -4097,7 +4099,7 @@
       <c r="J36" s="19"/>
       <c r="K36" s="19"/>
     </row>
-    <row r="37" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A37" s="2" t="s">
         <v>113</v>
       </c>
@@ -4125,7 +4127,7 @@
       <c r="J37" s="19"/>
       <c r="K37" s="19"/>
     </row>
-    <row r="38" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A38" s="2" t="s">
         <v>67</v>
       </c>
@@ -4153,7 +4155,7 @@
       <c r="J38" s="19"/>
       <c r="K38" s="19"/>
     </row>
-    <row r="39" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A39" s="2" t="s">
         <v>69</v>
       </c>
@@ -4181,7 +4183,7 @@
       <c r="J39" s="19"/>
       <c r="K39" s="19"/>
     </row>
-    <row r="40" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A40" s="2" t="s">
         <v>71</v>
       </c>
@@ -4209,7 +4211,7 @@
       <c r="J40" s="19"/>
       <c r="K40" s="19"/>
     </row>
-    <row r="41" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A41" s="2" t="s">
         <v>72</v>
       </c>
@@ -4237,7 +4239,7 @@
       <c r="J41" s="19"/>
       <c r="K41" s="19"/>
     </row>
-    <row r="42" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A42" s="2" t="s">
         <v>431</v>
       </c>
@@ -4265,7 +4267,7 @@
       <c r="J42" s="19"/>
       <c r="K42" s="19"/>
     </row>
-    <row r="43" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A43" s="2" t="s">
         <v>434</v>
       </c>
@@ -4293,7 +4295,7 @@
       <c r="J43" s="19"/>
       <c r="K43" s="19"/>
     </row>
-    <row r="44" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A44" s="2" t="s">
         <v>436</v>
       </c>
@@ -4321,7 +4323,7 @@
       <c r="J44" s="19"/>
       <c r="K44" s="19"/>
     </row>
-    <row r="45" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A45" s="2" t="s">
         <v>439</v>
       </c>
@@ -4349,7 +4351,7 @@
       <c r="J45" s="19"/>
       <c r="K45" s="19"/>
     </row>
-    <row r="46" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A46" s="2" t="s">
         <v>442</v>
       </c>
@@ -4377,7 +4379,7 @@
       <c r="J46" s="19"/>
       <c r="K46" s="19"/>
     </row>
-    <row r="47" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A47" s="2" t="s">
         <v>164</v>
       </c>
@@ -4405,7 +4407,7 @@
       <c r="J47" s="19"/>
       <c r="K47" s="19"/>
     </row>
-    <row r="48" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A48" s="2" t="s">
         <v>214</v>
       </c>
@@ -4433,7 +4435,7 @@
       <c r="J48" s="19"/>
       <c r="K48" s="19"/>
     </row>
-    <row r="49" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A49" s="2" t="s">
         <v>449</v>
       </c>
@@ -4461,7 +4463,7 @@
       <c r="J49" s="19"/>
       <c r="K49" s="19"/>
     </row>
-    <row r="50" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A50" s="2" t="s">
         <v>262</v>
       </c>
@@ -4489,7 +4491,7 @@
       <c r="J50" s="19"/>
       <c r="K50" s="19"/>
     </row>
-    <row r="51" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A51" s="2" t="s">
         <v>262</v>
       </c>
@@ -4517,7 +4519,7 @@
       <c r="J51" s="19"/>
       <c r="K51" s="19"/>
     </row>
-    <row r="52" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A52" s="2" t="s">
         <v>451</v>
       </c>
@@ -4545,7 +4547,7 @@
       <c r="J52" s="19"/>
       <c r="K52" s="19"/>
     </row>
-    <row r="53" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A53" s="2" t="s">
         <v>217</v>
       </c>
@@ -4573,7 +4575,7 @@
       <c r="J53" s="19"/>
       <c r="K53" s="19"/>
     </row>
-    <row r="54" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A54" s="2" t="s">
         <v>217</v>
       </c>
@@ -4601,7 +4603,7 @@
       <c r="J54" s="19"/>
       <c r="K54" s="19"/>
     </row>
-    <row r="55" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A55" s="2" t="s">
         <v>217</v>
       </c>
@@ -4629,7 +4631,7 @@
       <c r="J55" s="19"/>
       <c r="K55" s="19"/>
     </row>
-    <row r="56" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A56" s="2" t="s">
         <v>217</v>
       </c>
@@ -4657,7 +4659,7 @@
       <c r="J56" s="19"/>
       <c r="K56" s="19"/>
     </row>
-    <row r="57" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A57" s="2" t="s">
         <v>217</v>
       </c>
@@ -4685,7 +4687,7 @@
       <c r="J57" s="19"/>
       <c r="K57" s="19"/>
     </row>
-    <row r="58" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A58" s="2" t="s">
         <v>217</v>
       </c>
@@ -4713,7 +4715,7 @@
       <c r="J58" s="19"/>
       <c r="K58" s="19"/>
     </row>
-    <row r="59" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A59" s="2" t="s">
         <v>458</v>
       </c>
@@ -4741,7 +4743,7 @@
       <c r="J59" s="19"/>
       <c r="K59" s="19"/>
     </row>
-    <row r="60" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A60" s="2" t="s">
         <v>461</v>
       </c>
@@ -4769,7 +4771,7 @@
       <c r="J60" s="19"/>
       <c r="K60" s="19"/>
     </row>
-    <row r="61" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A61" s="2" t="s">
         <v>464</v>
       </c>
@@ -4797,7 +4799,7 @@
       <c r="J61" s="19"/>
       <c r="K61" s="19"/>
     </row>
-    <row r="62" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A62" s="2" t="s">
         <v>467</v>
       </c>
@@ -4825,7 +4827,7 @@
       <c r="J62" s="19"/>
       <c r="K62" s="19"/>
     </row>
-    <row r="63" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A63" s="2" t="s">
         <v>198</v>
       </c>
@@ -4853,7 +4855,7 @@
       <c r="J63" s="19"/>
       <c r="K63" s="19"/>
     </row>
-    <row r="64" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A64" s="2" t="s">
         <v>198</v>
       </c>
@@ -4881,7 +4883,7 @@
       <c r="J64" s="19"/>
       <c r="K64" s="19"/>
     </row>
-    <row r="65" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A65" s="2" t="s">
         <v>472</v>
       </c>
@@ -4909,7 +4911,7 @@
       <c r="J65" s="19"/>
       <c r="K65" s="19"/>
     </row>
-    <row r="66" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A66" s="2" t="s">
         <v>474</v>
       </c>
@@ -4937,7 +4939,7 @@
       <c r="J66" s="19"/>
       <c r="K66" s="19"/>
     </row>
-    <row r="67" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A67" s="2" t="s">
         <v>196</v>
       </c>
@@ -4965,7 +4967,7 @@
       <c r="J67" s="19"/>
       <c r="K67" s="19"/>
     </row>
-    <row r="68" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A68" s="2" t="s">
         <v>478</v>
       </c>
@@ -4993,7 +4995,7 @@
       <c r="J68" s="19"/>
       <c r="K68" s="19"/>
     </row>
-    <row r="69" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A69" s="2" t="s">
         <v>480</v>
       </c>
@@ -5021,7 +5023,7 @@
       <c r="J69" s="19"/>
       <c r="K69" s="19"/>
     </row>
-    <row r="70" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A70" s="2" t="s">
         <v>480</v>
       </c>
@@ -5049,7 +5051,7 @@
       <c r="J70" s="19"/>
       <c r="K70" s="19"/>
     </row>
-    <row r="71" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A71" s="2" t="s">
         <v>115</v>
       </c>
@@ -5077,7 +5079,7 @@
       <c r="J71" s="19"/>
       <c r="K71" s="19"/>
     </row>
-    <row r="72" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A72" s="2" t="s">
         <v>485</v>
       </c>
@@ -5105,7 +5107,7 @@
       <c r="J72" s="19"/>
       <c r="K72" s="19"/>
     </row>
-    <row r="73" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A73" s="2" t="s">
         <v>488</v>
       </c>
@@ -5133,7 +5135,7 @@
       <c r="J73" s="19"/>
       <c r="K73" s="19"/>
     </row>
-    <row r="74" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A74" s="2" t="s">
         <v>491</v>
       </c>
@@ -5161,7 +5163,7 @@
       <c r="J74" s="19"/>
       <c r="K74" s="19"/>
     </row>
-    <row r="75" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A75" s="2" t="s">
         <v>494</v>
       </c>
@@ -5189,7 +5191,7 @@
       <c r="J75" s="19"/>
       <c r="K75" s="19"/>
     </row>
-    <row r="76" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A76" s="2" t="s">
         <v>494</v>
       </c>
@@ -5217,7 +5219,7 @@
       <c r="J76" s="19"/>
       <c r="K76" s="19"/>
     </row>
-    <row r="77" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="77" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A77" s="2" t="s">
         <v>170</v>
       </c>
@@ -5245,7 +5247,7 @@
       <c r="J77" s="19"/>
       <c r="K77" s="19"/>
     </row>
-    <row r="78" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="78" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A78" s="2" t="s">
         <v>130</v>
       </c>
@@ -5273,7 +5275,7 @@
       <c r="J78" s="19"/>
       <c r="K78" s="19"/>
     </row>
-    <row r="79" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="79" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A79" s="2" t="s">
         <v>161</v>
       </c>
@@ -5301,7 +5303,7 @@
       <c r="J79" s="19"/>
       <c r="K79" s="19"/>
     </row>
-    <row r="80" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="80" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A80" s="2" t="s">
         <v>137</v>
       </c>
@@ -5329,7 +5331,7 @@
       <c r="J80" s="19"/>
       <c r="K80" s="19"/>
     </row>
-    <row r="81" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="81" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A81" s="2" t="s">
         <v>503</v>
       </c>
@@ -5357,7 +5359,7 @@
       <c r="J81" s="19"/>
       <c r="K81" s="19"/>
     </row>
-    <row r="82" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="82" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A82" s="2" t="s">
         <v>506</v>
       </c>
@@ -5385,7 +5387,7 @@
       <c r="J82" s="19"/>
       <c r="K82" s="19"/>
     </row>
-    <row r="83" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="83" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A83" s="2" t="s">
         <v>509</v>
       </c>
@@ -5413,7 +5415,7 @@
       <c r="J83" s="19"/>
       <c r="K83" s="19"/>
     </row>
-    <row r="84" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="84" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A84" s="2" t="s">
         <v>512</v>
       </c>
@@ -5441,7 +5443,7 @@
       <c r="J84" s="19"/>
       <c r="K84" s="19"/>
     </row>
-    <row r="85" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="85" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A85" s="2" t="s">
         <v>116</v>
       </c>
@@ -5469,7 +5471,7 @@
       <c r="J85" s="19"/>
       <c r="K85" s="19"/>
     </row>
-    <row r="86" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A86" s="2" t="s">
         <v>516</v>
       </c>
@@ -5497,7 +5499,7 @@
       <c r="J86" s="19"/>
       <c r="K86" s="19"/>
     </row>
-    <row r="87" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="87" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A87" s="2" t="s">
         <v>519</v>
       </c>
@@ -5525,7 +5527,7 @@
       <c r="J87" s="19"/>
       <c r="K87" s="19"/>
     </row>
-    <row r="88" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="88" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A88" s="2" t="s">
         <v>519</v>
       </c>
@@ -5553,7 +5555,7 @@
       <c r="J88" s="19"/>
       <c r="K88" s="19"/>
     </row>
-    <row r="89" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="89" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A89" s="2" t="s">
         <v>519</v>
       </c>
@@ -5581,7 +5583,7 @@
       <c r="J89" s="19"/>
       <c r="K89" s="19"/>
     </row>
-    <row r="90" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="90" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A90" s="2" t="s">
         <v>522</v>
       </c>
@@ -5609,7 +5611,7 @@
       <c r="J90" s="19"/>
       <c r="K90" s="19"/>
     </row>
-    <row r="91" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="91" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A91" s="2" t="s">
         <v>525</v>
       </c>
@@ -5637,7 +5639,7 @@
       <c r="J91" s="19"/>
       <c r="K91" s="19"/>
     </row>
-    <row r="92" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="92" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A92" s="2" t="s">
         <v>117</v>
       </c>
@@ -5665,7 +5667,7 @@
       <c r="J92" s="19"/>
       <c r="K92" s="19"/>
     </row>
-    <row r="93" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="93" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A93" s="2" t="s">
         <v>529</v>
       </c>
@@ -5693,7 +5695,7 @@
       <c r="J93" s="19"/>
       <c r="K93" s="19"/>
     </row>
-    <row r="94" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="94" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A94" s="2" t="s">
         <v>529</v>
       </c>
@@ -5721,7 +5723,7 @@
       <c r="J94" s="19"/>
       <c r="K94" s="19"/>
     </row>
-    <row r="95" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="95" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A95" s="2" t="s">
         <v>529</v>
       </c>
@@ -5749,7 +5751,7 @@
       <c r="J95" s="19"/>
       <c r="K95" s="19"/>
     </row>
-    <row r="96" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="96" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A96" s="2" t="s">
         <v>531</v>
       </c>
@@ -5777,7 +5779,7 @@
       <c r="J96" s="19"/>
       <c r="K96" s="19"/>
     </row>
-    <row r="97" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="97" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A97" s="2" t="s">
         <v>536</v>
       </c>
@@ -5805,7 +5807,7 @@
       <c r="J97" s="19"/>
       <c r="K97" s="19"/>
     </row>
-    <row r="98" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="98" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A98" s="2" t="s">
         <v>536</v>
       </c>
@@ -5833,7 +5835,7 @@
       <c r="J98" s="19"/>
       <c r="K98" s="19"/>
     </row>
-    <row r="99" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A99" s="2" t="s">
         <v>534</v>
       </c>
@@ -5861,7 +5863,7 @@
       <c r="J99" s="19"/>
       <c r="K99" s="19"/>
     </row>
-    <row r="100" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="100" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A100" s="2" t="s">
         <v>267</v>
       </c>
@@ -5889,7 +5891,7 @@
       <c r="J100" s="19"/>
       <c r="K100" s="19"/>
     </row>
-    <row r="101" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A101" s="2" t="s">
         <v>267</v>
       </c>
@@ -5917,7 +5919,7 @@
       <c r="J101" s="19"/>
       <c r="K101" s="19"/>
     </row>
-    <row r="102" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A102" s="2" t="s">
         <v>540</v>
       </c>
@@ -5945,7 +5947,7 @@
       <c r="J102" s="19"/>
       <c r="K102" s="19"/>
     </row>
-    <row r="103" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A103" s="2" t="s">
         <v>540</v>
       </c>
@@ -5973,7 +5975,7 @@
       <c r="J103" s="19"/>
       <c r="K103" s="19"/>
     </row>
-    <row r="104" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A104" s="2" t="s">
         <v>540</v>
       </c>
@@ -6001,7 +6003,7 @@
       <c r="J104" s="19"/>
       <c r="K104" s="19"/>
     </row>
-    <row r="105" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A105" s="2" t="s">
         <v>543</v>
       </c>
@@ -6029,7 +6031,7 @@
       <c r="J105" s="19"/>
       <c r="K105" s="19"/>
     </row>
-    <row r="106" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A106" s="2" t="s">
         <v>543</v>
       </c>
@@ -6057,7 +6059,7 @@
       <c r="J106" s="19"/>
       <c r="K106" s="19"/>
     </row>
-    <row r="107" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A107" s="2" t="s">
         <v>545</v>
       </c>
@@ -6085,7 +6087,7 @@
       <c r="J107" s="19"/>
       <c r="K107" s="19"/>
     </row>
-    <row r="108" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A108" s="2" t="s">
         <v>548</v>
       </c>
@@ -6113,7 +6115,7 @@
       <c r="J108" s="19"/>
       <c r="K108" s="19"/>
     </row>
-    <row r="109" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A109" s="2" t="s">
         <v>805</v>
       </c>
@@ -6141,7 +6143,7 @@
       <c r="J109" s="19"/>
       <c r="K109" s="19"/>
     </row>
-    <row r="110" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A110" s="2" t="s">
         <v>167</v>
       </c>
@@ -6169,7 +6171,7 @@
       <c r="J110" s="19"/>
       <c r="K110" s="19"/>
     </row>
-    <row r="111" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A111" s="2" t="s">
         <v>554</v>
       </c>
@@ -6197,7 +6199,7 @@
       <c r="J111" s="19"/>
       <c r="K111" s="19"/>
     </row>
-    <row r="112" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A112" s="2" t="s">
         <v>295</v>
       </c>
@@ -6225,7 +6227,7 @@
       <c r="J112" s="19"/>
       <c r="K112" s="19"/>
     </row>
-    <row r="113" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="113" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A113" s="2" t="s">
         <v>558</v>
       </c>
@@ -6253,7 +6255,7 @@
       <c r="J113" s="19"/>
       <c r="K113" s="19"/>
     </row>
-    <row r="114" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="114" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A114" s="2" t="s">
         <v>560</v>
       </c>
@@ -6281,7 +6283,7 @@
       <c r="J114" s="19"/>
       <c r="K114" s="19"/>
     </row>
-    <row r="115" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="115" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A115" s="2" t="s">
         <v>110</v>
       </c>
@@ -6309,7 +6311,7 @@
       <c r="J115" s="19"/>
       <c r="K115" s="19"/>
     </row>
-    <row r="116" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="116" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A116" s="2" t="s">
         <v>353</v>
       </c>
@@ -6337,7 +6339,7 @@
       <c r="J116" s="19"/>
       <c r="K116" s="19"/>
     </row>
-    <row r="117" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="117" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A117" s="2" t="s">
         <v>564</v>
       </c>
@@ -6365,7 +6367,7 @@
       <c r="J117" s="19"/>
       <c r="K117" s="19"/>
     </row>
-    <row r="118" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="118" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A118" s="2" t="s">
         <v>564</v>
       </c>
@@ -6393,7 +6395,7 @@
       <c r="J118" s="19"/>
       <c r="K118" s="19"/>
     </row>
-    <row r="119" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="119" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A119" s="2" t="s">
         <v>350</v>
       </c>
@@ -6421,7 +6423,7 @@
       <c r="J119" s="19"/>
       <c r="K119" s="19"/>
     </row>
-    <row r="120" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="120" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A120" s="2" t="s">
         <v>568</v>
       </c>
@@ -6449,7 +6451,7 @@
       <c r="J120" s="19"/>
       <c r="K120" s="19"/>
     </row>
-    <row r="121" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="121" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A121" s="2" t="s">
         <v>568</v>
       </c>
@@ -6477,7 +6479,7 @@
       <c r="J121" s="19"/>
       <c r="K121" s="19"/>
     </row>
-    <row r="122" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="122" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A122" s="2" t="s">
         <v>800</v>
       </c>
@@ -6505,7 +6507,7 @@
       <c r="J122" s="19"/>
       <c r="K122" s="19"/>
     </row>
-    <row r="123" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="123" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A123" s="2" t="s">
         <v>121</v>
       </c>
@@ -6533,7 +6535,7 @@
       <c r="J123" s="19"/>
       <c r="K123" s="19"/>
     </row>
-    <row r="124" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="124" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A124" s="2" t="s">
         <v>572</v>
       </c>
@@ -6561,7 +6563,7 @@
       <c r="J124" s="19"/>
       <c r="K124" s="19"/>
     </row>
-    <row r="125" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A125" s="2" t="s">
         <v>572</v>
       </c>
@@ -6589,7 +6591,7 @@
       <c r="J125" s="19"/>
       <c r="K125" s="19"/>
     </row>
-    <row r="126" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="126" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A126" s="2" t="s">
         <v>575</v>
       </c>
@@ -6619,7 +6621,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="127" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="127" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A127" s="2" t="s">
         <v>135</v>
       </c>
@@ -6647,7 +6649,7 @@
       <c r="J127" s="19"/>
       <c r="K127" s="19"/>
     </row>
-    <row r="128" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="128" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A128" s="2" t="s">
         <v>231</v>
       </c>
@@ -6675,7 +6677,7 @@
       <c r="J128" s="19"/>
       <c r="K128" s="19"/>
     </row>
-    <row r="129" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="129" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A129" s="2" t="s">
         <v>581</v>
       </c>
@@ -6703,7 +6705,7 @@
       <c r="J129" s="19"/>
       <c r="K129" s="19"/>
     </row>
-    <row r="130" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="130" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A130" s="2" t="s">
         <v>581</v>
       </c>
@@ -6731,7 +6733,7 @@
       <c r="J130" s="19"/>
       <c r="K130" s="19"/>
     </row>
-    <row r="131" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="131" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A131" s="2" t="s">
         <v>584</v>
       </c>
@@ -6759,7 +6761,7 @@
       <c r="J131" s="19"/>
       <c r="K131" s="19"/>
     </row>
-    <row r="132" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="132" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A132" s="2" t="s">
         <v>587</v>
       </c>
@@ -6787,7 +6789,7 @@
       <c r="J132" s="19"/>
       <c r="K132" s="19"/>
     </row>
-    <row r="133" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="133" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A133" s="2" t="s">
         <v>590</v>
       </c>
@@ -6815,7 +6817,7 @@
       <c r="J133" s="19"/>
       <c r="K133" s="19"/>
     </row>
-    <row r="134" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="134" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A134" s="2" t="s">
         <v>593</v>
       </c>
@@ -6843,7 +6845,7 @@
       <c r="J134" s="19"/>
       <c r="K134" s="19"/>
     </row>
-    <row r="135" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="135" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A135" s="2" t="s">
         <v>145</v>
       </c>
@@ -6871,7 +6873,7 @@
       <c r="J135" s="19"/>
       <c r="K135" s="19"/>
     </row>
-    <row r="136" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="136" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A136" s="2" t="s">
         <v>596</v>
       </c>
@@ -6899,7 +6901,7 @@
       <c r="J136" s="19"/>
       <c r="K136" s="19"/>
     </row>
-    <row r="137" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="137" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A137" s="2" t="s">
         <v>598</v>
       </c>
@@ -6927,7 +6929,7 @@
       <c r="J137" s="19"/>
       <c r="K137" s="19"/>
     </row>
-    <row r="138" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A138" s="2" t="s">
         <v>601</v>
       </c>
@@ -6955,7 +6957,7 @@
       <c r="J138" s="19"/>
       <c r="K138" s="19"/>
     </row>
-    <row r="139" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="139" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A139" s="2" t="s">
         <v>604</v>
       </c>
@@ -6983,7 +6985,7 @@
       <c r="J139" s="19"/>
       <c r="K139" s="19"/>
     </row>
-    <row r="140" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="140" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A140" s="2" t="s">
         <v>607</v>
       </c>
@@ -7011,7 +7013,7 @@
       <c r="J140" s="19"/>
       <c r="K140" s="19"/>
     </row>
-    <row r="141" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="141" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A141" s="2" t="s">
         <v>610</v>
       </c>
@@ -7039,7 +7041,7 @@
       <c r="J141" s="19"/>
       <c r="K141" s="19"/>
     </row>
-    <row r="142" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="142" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A142" s="2" t="s">
         <v>613</v>
       </c>
@@ -7067,7 +7069,7 @@
       <c r="J142" s="19"/>
       <c r="K142" s="19"/>
     </row>
-    <row r="143" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="143" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A143" s="2" t="s">
         <v>616</v>
       </c>
@@ -7095,7 +7097,7 @@
       <c r="J143" s="19"/>
       <c r="K143" s="19"/>
     </row>
-    <row r="144" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="144" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A144" s="2" t="s">
         <v>619</v>
       </c>
@@ -7123,7 +7125,7 @@
       <c r="J144" s="19"/>
       <c r="K144" s="19"/>
     </row>
-    <row r="145" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="145" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A145" s="2" t="s">
         <v>622</v>
       </c>
@@ -7151,7 +7153,7 @@
       <c r="J145" s="19"/>
       <c r="K145" s="19"/>
     </row>
-    <row r="146" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="146" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A146" s="2" t="s">
         <v>622</v>
       </c>
@@ -7179,7 +7181,7 @@
       <c r="J146" s="19"/>
       <c r="K146" s="19"/>
     </row>
-    <row r="147" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A147" s="2" t="s">
         <v>624</v>
       </c>
@@ -7207,7 +7209,7 @@
       <c r="J147" s="19"/>
       <c r="K147" s="19"/>
     </row>
-    <row r="148" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A148" s="2" t="s">
         <v>627</v>
       </c>
@@ -7235,7 +7237,7 @@
       <c r="J148" s="19"/>
       <c r="K148" s="19"/>
     </row>
-    <row r="149" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A149" s="2" t="s">
         <v>630</v>
       </c>
@@ -7263,7 +7265,7 @@
       <c r="J149" s="19"/>
       <c r="K149" s="19"/>
     </row>
-    <row r="150" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A150" s="2" t="s">
         <v>633</v>
       </c>
@@ -7291,7 +7293,7 @@
       <c r="J150" s="19"/>
       <c r="K150" s="19"/>
     </row>
-    <row r="151" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A151" s="2" t="s">
         <v>636</v>
       </c>
@@ -7319,7 +7321,7 @@
       <c r="J151" s="19"/>
       <c r="K151" s="19"/>
     </row>
-    <row r="152" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A152" s="2" t="s">
         <v>639</v>
       </c>
@@ -7351,7 +7353,7 @@
       <c r="J152" s="19"/>
       <c r="K152" s="19"/>
     </row>
-    <row r="153" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A153" s="2" t="s">
         <v>202</v>
       </c>
@@ -7379,7 +7381,7 @@
       <c r="J153" s="19"/>
       <c r="K153" s="19"/>
     </row>
-    <row r="154" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A154" s="2" t="s">
         <v>122</v>
       </c>
@@ -7407,7 +7409,7 @@
       <c r="J154" s="19"/>
       <c r="K154" s="19"/>
     </row>
-    <row r="155" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A155" s="2" t="s">
         <v>122</v>
       </c>
@@ -7435,7 +7437,7 @@
       <c r="J155" s="19"/>
       <c r="K155" s="19"/>
     </row>
-    <row r="156" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A156" s="2" t="s">
         <v>103</v>
       </c>
@@ -7463,7 +7465,7 @@
       <c r="J156" s="19"/>
       <c r="K156" s="19"/>
     </row>
-    <row r="157" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A157" s="2" t="s">
         <v>105</v>
       </c>
@@ -7491,7 +7493,7 @@
       <c r="J157" s="19"/>
       <c r="K157" s="19"/>
     </row>
-    <row r="158" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A158" s="2" t="s">
         <v>107</v>
       </c>
@@ -7519,7 +7521,7 @@
       <c r="J158" s="19"/>
       <c r="K158" s="19"/>
     </row>
-    <row r="159" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A159" s="2" t="s">
         <v>111</v>
       </c>
@@ -7547,7 +7549,7 @@
       <c r="J159" s="19"/>
       <c r="K159" s="19"/>
     </row>
-    <row r="160" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A160" s="2" t="s">
         <v>651</v>
       </c>
@@ -7575,7 +7577,7 @@
       <c r="J160" s="19"/>
       <c r="K160" s="19"/>
     </row>
-    <row r="161" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="161" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A161" s="2" t="s">
         <v>654</v>
       </c>
@@ -7603,7 +7605,7 @@
       <c r="J161" s="19"/>
       <c r="K161" s="19"/>
     </row>
-    <row r="162" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="162" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A162" s="2" t="s">
         <v>148</v>
       </c>
@@ -7631,7 +7633,7 @@
       <c r="J162" s="19"/>
       <c r="K162" s="19"/>
     </row>
-    <row r="163" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="163" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A163" s="2" t="s">
         <v>134</v>
       </c>
@@ -7657,11 +7659,9 @@
       <c r="H163" s="19"/>
       <c r="I163" s="19"/>
       <c r="J163" s="19"/>
-      <c r="K163" s="19" t="s">
-        <v>825</v>
-      </c>
-    </row>
-    <row r="164" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K163" s="19"/>
+    </row>
+    <row r="164" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A164" s="2" t="s">
         <v>282</v>
       </c>
@@ -7689,7 +7689,7 @@
       <c r="J164" s="19"/>
       <c r="K164" s="19"/>
     </row>
-    <row r="165" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="165" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A165" s="2" t="s">
         <v>127</v>
       </c>
@@ -7717,7 +7717,7 @@
       <c r="J165" s="19"/>
       <c r="K165" s="19"/>
     </row>
-    <row r="166" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="166" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A166" s="2" t="s">
         <v>127</v>
       </c>
@@ -7745,7 +7745,7 @@
       <c r="J166" s="19"/>
       <c r="K166" s="19"/>
     </row>
-    <row r="167" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="167" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A167" s="2" t="s">
         <v>158</v>
       </c>
@@ -7773,7 +7773,7 @@
       <c r="J167" s="19"/>
       <c r="K167" s="19"/>
     </row>
-    <row r="168" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="168" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A168" s="2" t="s">
         <v>177</v>
       </c>
@@ -7801,7 +7801,7 @@
       <c r="J168" s="19"/>
       <c r="K168" s="19"/>
     </row>
-    <row r="169" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="169" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A169" s="2" t="s">
         <v>132</v>
       </c>
@@ -7829,7 +7829,7 @@
       <c r="J169" s="19"/>
       <c r="K169" s="19"/>
     </row>
-    <row r="170" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="170" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A170" s="2" t="s">
         <v>131</v>
       </c>
@@ -7857,7 +7857,7 @@
       <c r="J170" s="19"/>
       <c r="K170" s="19"/>
     </row>
-    <row r="171" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="171" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A171" s="2" t="s">
         <v>141</v>
       </c>
@@ -7885,7 +7885,7 @@
       <c r="J171" s="19"/>
       <c r="K171" s="19"/>
     </row>
-    <row r="172" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="172" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A172" s="2" t="s">
         <v>142</v>
       </c>
@@ -7913,7 +7913,7 @@
       <c r="J172" s="19"/>
       <c r="K172" s="19"/>
     </row>
-    <row r="173" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="173" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A173" s="2" t="s">
         <v>228</v>
       </c>
@@ -7941,7 +7941,7 @@
       <c r="J173" s="19"/>
       <c r="K173" s="19"/>
     </row>
-    <row r="174" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="174" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A174" s="2" t="s">
         <v>230</v>
       </c>
@@ -7969,7 +7969,7 @@
       <c r="J174" s="19"/>
       <c r="K174" s="19"/>
     </row>
-    <row r="175" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="175" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A175" s="2" t="s">
         <v>147</v>
       </c>
@@ -7997,7 +7997,7 @@
       <c r="J175" s="19"/>
       <c r="K175" s="19"/>
     </row>
-    <row r="176" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="176" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A176" s="2" t="s">
         <v>151</v>
       </c>
@@ -8025,7 +8025,7 @@
       <c r="J176" s="19"/>
       <c r="K176" s="19"/>
     </row>
-    <row r="177" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A177" s="2" t="s">
         <v>681</v>
       </c>
@@ -8053,7 +8053,7 @@
       <c r="J177" s="19"/>
       <c r="K177" s="19"/>
     </row>
-    <row r="178" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="178" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A178" s="2" t="s">
         <v>154</v>
       </c>
@@ -8081,7 +8081,7 @@
       <c r="J178" s="19"/>
       <c r="K178" s="19"/>
     </row>
-    <row r="179" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="179" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A179" s="2" t="s">
         <v>156</v>
       </c>
@@ -8109,7 +8109,7 @@
       <c r="J179" s="19"/>
       <c r="K179" s="19"/>
     </row>
-    <row r="180" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="180" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A180" s="2" t="s">
         <v>168</v>
       </c>
@@ -8137,7 +8137,7 @@
       <c r="J180" s="19"/>
       <c r="K180" s="19"/>
     </row>
-    <row r="181" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="181" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A181" s="2" t="s">
         <v>163</v>
       </c>
@@ -8165,7 +8165,7 @@
       <c r="J181" s="19"/>
       <c r="K181" s="19"/>
     </row>
-    <row r="182" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="182" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A182" s="2" t="s">
         <v>374</v>
       </c>
@@ -8193,7 +8193,7 @@
       <c r="J182" s="19"/>
       <c r="K182" s="19"/>
     </row>
-    <row r="183" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="183" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A183" s="2" t="s">
         <v>173</v>
       </c>
@@ -8221,7 +8221,7 @@
       <c r="J183" s="19"/>
       <c r="K183" s="19"/>
     </row>
-    <row r="184" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="184" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A184" s="2" t="s">
         <v>173</v>
       </c>
@@ -8249,7 +8249,7 @@
       <c r="J184" s="19"/>
       <c r="K184" s="19"/>
     </row>
-    <row r="185" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="185" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A185" s="2" t="s">
         <v>175</v>
       </c>
@@ -8277,7 +8277,7 @@
       <c r="J185" s="19"/>
       <c r="K185" s="19"/>
     </row>
-    <row r="186" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="186" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A186" s="2" t="s">
         <v>175</v>
       </c>
@@ -8305,7 +8305,7 @@
       <c r="J186" s="19"/>
       <c r="K186" s="19"/>
     </row>
-    <row r="187" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="187" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A187" s="2" t="s">
         <v>175</v>
       </c>
@@ -8333,7 +8333,7 @@
       <c r="J187" s="19"/>
       <c r="K187" s="19"/>
     </row>
-    <row r="188" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="188" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A188" s="2" t="s">
         <v>179</v>
       </c>
@@ -8361,7 +8361,7 @@
       <c r="J188" s="19"/>
       <c r="K188" s="19"/>
     </row>
-    <row r="189" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="189" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A189" s="2" t="s">
         <v>696</v>
       </c>
@@ -8387,11 +8387,9 @@
       <c r="H189" s="19"/>
       <c r="I189" s="19"/>
       <c r="J189" s="19"/>
-      <c r="K189" s="19" t="s">
-        <v>825</v>
-      </c>
-    </row>
-    <row r="190" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="K189" s="19"/>
+    </row>
+    <row r="190" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A190" s="2" t="s">
         <v>298</v>
       </c>
@@ -8419,7 +8417,7 @@
       <c r="J190" s="19"/>
       <c r="K190" s="19"/>
     </row>
-    <row r="191" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="191" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A191" s="2" t="s">
         <v>797</v>
       </c>
@@ -8447,7 +8445,7 @@
       <c r="J191" s="19"/>
       <c r="K191" s="19"/>
     </row>
-    <row r="192" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="192" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A192" s="2" t="s">
         <v>185</v>
       </c>
@@ -8475,7 +8473,7 @@
       <c r="J192" s="19"/>
       <c r="K192" s="19"/>
     </row>
-    <row r="193" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="193" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A193" s="2" t="s">
         <v>185</v>
       </c>
@@ -8503,7 +8501,7 @@
       <c r="J193" s="19"/>
       <c r="K193" s="19"/>
     </row>
-    <row r="194" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="194" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A194" s="2" t="s">
         <v>183</v>
       </c>
@@ -8531,7 +8529,7 @@
       <c r="J194" s="19"/>
       <c r="K194" s="19"/>
     </row>
-    <row r="195" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="195" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A195" s="2" t="s">
         <v>703</v>
       </c>
@@ -8559,7 +8557,7 @@
       <c r="J195" s="19"/>
       <c r="K195" s="19"/>
     </row>
-    <row r="196" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="196" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A196" s="2" t="s">
         <v>705</v>
       </c>
@@ -8587,7 +8585,7 @@
       <c r="J196" s="19"/>
       <c r="K196" s="19"/>
     </row>
-    <row r="197" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="197" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A197" s="2" t="s">
         <v>188</v>
       </c>
@@ -8615,7 +8613,7 @@
       <c r="J197" s="19"/>
       <c r="K197" s="19"/>
     </row>
-    <row r="198" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="198" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A198" s="2" t="s">
         <v>191</v>
       </c>
@@ -8643,7 +8641,7 @@
       <c r="J198" s="19"/>
       <c r="K198" s="19"/>
     </row>
-    <row r="199" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="199" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A199" s="2" t="s">
         <v>711</v>
       </c>
@@ -8671,7 +8669,7 @@
       <c r="J199" s="19"/>
       <c r="K199" s="19"/>
     </row>
-    <row r="200" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="200" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A200" s="2" t="s">
         <v>219</v>
       </c>
@@ -8699,7 +8697,7 @@
       <c r="J200" s="19"/>
       <c r="K200" s="19"/>
     </row>
-    <row r="201" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="201" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A201" s="2" t="s">
         <v>713</v>
       </c>
@@ -8727,7 +8725,7 @@
       <c r="J201" s="19"/>
       <c r="K201" s="19"/>
     </row>
-    <row r="202" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="202" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A202" s="2" t="s">
         <v>716</v>
       </c>
@@ -8757,7 +8755,7 @@
         <v>825</v>
       </c>
     </row>
-    <row r="203" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A203" s="2" t="s">
         <v>359</v>
       </c>
@@ -8785,7 +8783,7 @@
       <c r="J203" s="19"/>
       <c r="K203" s="19"/>
     </row>
-    <row r="204" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="204" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A204" s="2" t="s">
         <v>204</v>
       </c>
@@ -8813,7 +8811,7 @@
       <c r="J204" s="19"/>
       <c r="K204" s="19"/>
     </row>
-    <row r="205" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="205" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A205" s="2" t="s">
         <v>206</v>
       </c>
@@ -8841,7 +8839,7 @@
       <c r="J205" s="19"/>
       <c r="K205" s="19"/>
     </row>
-    <row r="206" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="206" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A206" s="2" t="s">
         <v>240</v>
       </c>
@@ -8869,7 +8867,7 @@
       <c r="J206" s="19"/>
       <c r="K206" s="19"/>
     </row>
-    <row r="207" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="207" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A207" s="2" t="s">
         <v>212</v>
       </c>
@@ -8897,7 +8895,7 @@
       <c r="J207" s="19"/>
       <c r="K207" s="19"/>
     </row>
-    <row r="208" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="208" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A208" s="2" t="s">
         <v>226</v>
       </c>
@@ -8925,7 +8923,7 @@
       <c r="J208" s="19"/>
       <c r="K208" s="19"/>
     </row>
-    <row r="209" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="209" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A209" s="2" t="s">
         <v>221</v>
       </c>
@@ -8953,7 +8951,7 @@
       <c r="J209" s="19"/>
       <c r="K209" s="19"/>
     </row>
-    <row r="210" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="210" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A210" s="2" t="s">
         <v>221</v>
       </c>
@@ -8981,7 +8979,7 @@
       <c r="J210" s="19"/>
       <c r="K210" s="19"/>
     </row>
-    <row r="211" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="211" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A211" s="2" t="s">
         <v>221</v>
       </c>
@@ -9009,7 +9007,7 @@
       <c r="J211" s="19"/>
       <c r="K211" s="19"/>
     </row>
-    <row r="212" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="212" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A212" s="2" t="s">
         <v>221</v>
       </c>
@@ -9037,7 +9035,7 @@
       <c r="J212" s="19"/>
       <c r="K212" s="19"/>
     </row>
-    <row r="213" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="213" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A213" s="2" t="s">
         <v>221</v>
       </c>
@@ -9065,7 +9063,7 @@
       <c r="J213" s="19"/>
       <c r="K213" s="19"/>
     </row>
-    <row r="214" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="214" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A214" s="2" t="s">
         <v>732</v>
       </c>
@@ -9093,7 +9091,7 @@
       <c r="J214" s="19"/>
       <c r="K214" s="19"/>
     </row>
-    <row r="215" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="215" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A215" s="2" t="s">
         <v>232</v>
       </c>
@@ -9121,7 +9119,7 @@
       <c r="J215" s="19"/>
       <c r="K215" s="19"/>
     </row>
-    <row r="216" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A216" s="2" t="s">
         <v>242</v>
       </c>
@@ -9149,7 +9147,7 @@
       <c r="J216" s="19"/>
       <c r="K216" s="19"/>
     </row>
-    <row r="217" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="217" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A217" s="2" t="s">
         <v>247</v>
       </c>
@@ -9177,7 +9175,7 @@
       <c r="J217" s="19"/>
       <c r="K217" s="19"/>
     </row>
-    <row r="218" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="218" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A218" s="2" t="s">
         <v>740</v>
       </c>
@@ -9205,7 +9203,7 @@
       <c r="J218" s="19"/>
       <c r="K218" s="19"/>
     </row>
-    <row r="219" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="219" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A219" s="2" t="s">
         <v>251</v>
       </c>
@@ -9233,7 +9231,7 @@
       <c r="J219" s="19"/>
       <c r="K219" s="19"/>
     </row>
-    <row r="220" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="220" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A220" s="2" t="s">
         <v>276</v>
       </c>
@@ -9261,7 +9259,7 @@
       <c r="J220" s="19"/>
       <c r="K220" s="19"/>
     </row>
-    <row r="221" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="221" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A221" s="2" t="s">
         <v>746</v>
       </c>
@@ -9289,7 +9287,7 @@
       <c r="J221" s="19"/>
       <c r="K221" s="19"/>
     </row>
-    <row r="222" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="222" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A222" s="2" t="s">
         <v>257</v>
       </c>
@@ -9317,7 +9315,7 @@
       <c r="J222" s="19"/>
       <c r="K222" s="19"/>
     </row>
-    <row r="223" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="223" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A223" s="2" t="s">
         <v>748</v>
       </c>
@@ -9345,7 +9343,7 @@
       <c r="J223" s="19"/>
       <c r="K223" s="19"/>
     </row>
-    <row r="224" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="224" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A224" s="2" t="s">
         <v>263</v>
       </c>
@@ -9373,7 +9371,7 @@
       <c r="J224" s="19"/>
       <c r="K224" s="19"/>
     </row>
-    <row r="225" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="225" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A225" s="2" t="s">
         <v>260</v>
       </c>
@@ -9401,7 +9399,7 @@
       <c r="J225" s="19"/>
       <c r="K225" s="19"/>
     </row>
-    <row r="226" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="226" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A226" s="2" t="s">
         <v>264</v>
       </c>
@@ -9429,7 +9427,7 @@
       <c r="J226" s="19"/>
       <c r="K226" s="19"/>
     </row>
-    <row r="227" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="227" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A227" s="2" t="s">
         <v>269</v>
       </c>
@@ -9457,7 +9455,7 @@
       <c r="J227" s="19"/>
       <c r="K227" s="19"/>
     </row>
-    <row r="228" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="228" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A228" s="2" t="s">
         <v>270</v>
       </c>
@@ -9485,7 +9483,7 @@
       <c r="J228" s="19"/>
       <c r="K228" s="19"/>
     </row>
-    <row r="229" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A229" s="2" t="s">
         <v>270</v>
       </c>
@@ -9513,7 +9511,7 @@
       <c r="J229" s="19"/>
       <c r="K229" s="19"/>
     </row>
-    <row r="230" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="230" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A230" s="2" t="s">
         <v>279</v>
       </c>
@@ -9541,7 +9539,7 @@
       <c r="J230" s="19"/>
       <c r="K230" s="19"/>
     </row>
-    <row r="231" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="231" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A231" s="2" t="s">
         <v>278</v>
       </c>
@@ -9569,7 +9567,7 @@
       <c r="J231" s="19"/>
       <c r="K231" s="19"/>
     </row>
-    <row r="232" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="232" spans="1:11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A232" s="2" t="s">
         <v>284</v>
       </c>
@@ -9597,7 +9595,7 @@
       <c r="J232" s="20"/>
       <c r="K232" s="20"/>
     </row>
-    <row r="233" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="233" spans="1:11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A233" s="2" t="s">
         <v>765</v>
       </c>
@@ -9625,7 +9623,7 @@
       <c r="J233" s="20"/>
       <c r="K233" s="20"/>
     </row>
-    <row r="234" spans="1:11" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="234" spans="1:11" customFormat="1" x14ac:dyDescent="0.35">
       <c r="A234" s="2" t="s">
         <v>288</v>
       </c>
@@ -9653,7 +9651,7 @@
       <c r="J234" s="20"/>
       <c r="K234" s="20"/>
     </row>
-    <row r="235" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="235" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A235" s="2" t="s">
         <v>287</v>
       </c>
@@ -9681,7 +9679,7 @@
       <c r="J235" s="19"/>
       <c r="K235" s="19"/>
     </row>
-    <row r="236" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="236" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A236" s="2" t="s">
         <v>289</v>
       </c>
@@ -9709,7 +9707,7 @@
       <c r="J236" s="19"/>
       <c r="K236" s="19"/>
     </row>
-    <row r="237" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="237" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A237" s="2" t="s">
         <v>290</v>
       </c>
@@ -9737,7 +9735,7 @@
       <c r="J237" s="19"/>
       <c r="K237" s="19"/>
     </row>
-    <row r="238" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="238" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A238" s="2" t="s">
         <v>774</v>
       </c>
@@ -9765,7 +9763,7 @@
       <c r="J238" s="19"/>
       <c r="K238" s="19"/>
     </row>
-    <row r="239" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="239" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A239" s="2" t="s">
         <v>303</v>
       </c>
@@ -9793,7 +9791,7 @@
       <c r="J239" s="19"/>
       <c r="K239" s="19"/>
     </row>
-    <row r="240" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="240" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A240" s="2" t="s">
         <v>304</v>
       </c>
@@ -9821,7 +9819,7 @@
       <c r="J240" s="19"/>
       <c r="K240" s="19"/>
     </row>
-    <row r="241" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="241" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A241" s="2" t="s">
         <v>305</v>
       </c>
@@ -9849,7 +9847,7 @@
       <c r="J241" s="19"/>
       <c r="K241" s="19"/>
     </row>
-    <row r="242" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A242" s="2" t="s">
         <v>300</v>
       </c>
@@ -9877,7 +9875,7 @@
       <c r="J242" s="19"/>
       <c r="K242" s="19"/>
     </row>
-    <row r="243" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="243" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A243" s="2" t="s">
         <v>348</v>
       </c>
@@ -9905,7 +9903,7 @@
       <c r="J243" s="19"/>
       <c r="K243" s="19"/>
     </row>
-    <row r="244" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="244" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A244" s="2" t="s">
         <v>357</v>
       </c>
@@ -9933,7 +9931,7 @@
       <c r="J244" s="19"/>
       <c r="K244" s="19"/>
     </row>
-    <row r="245" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="245" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A245" s="2" t="s">
         <v>351</v>
       </c>
@@ -9961,7 +9959,7 @@
       <c r="J245" s="19"/>
       <c r="K245" s="19"/>
     </row>
-    <row r="246" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="246" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A246" s="2" t="s">
         <v>361</v>
       </c>
@@ -9989,7 +9987,7 @@
       <c r="J246" s="19"/>
       <c r="K246" s="19"/>
     </row>
-    <row r="247" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="247" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A247" s="2" t="s">
         <v>365</v>
       </c>
@@ -10017,7 +10015,7 @@
       <c r="J247" s="19"/>
       <c r="K247" s="19"/>
     </row>
-    <row r="248" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="248" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A248" s="2" t="s">
         <v>363</v>
       </c>
@@ -10045,7 +10043,7 @@
       <c r="J248" s="19"/>
       <c r="K248" s="19"/>
     </row>
-    <row r="249" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="249" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A249" s="2" t="s">
         <v>355</v>
       </c>
@@ -10073,7 +10071,7 @@
       <c r="J249" s="19"/>
       <c r="K249" s="19"/>
     </row>
-    <row r="250" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="250" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A250" s="2" t="s">
         <v>368</v>
       </c>
@@ -10101,7 +10099,7 @@
       <c r="J250" s="19"/>
       <c r="K250" s="19"/>
     </row>
-    <row r="251" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="251" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A251" s="2" t="s">
         <v>367</v>
       </c>
@@ -10129,7 +10127,7 @@
       <c r="J251" s="19"/>
       <c r="K251" s="19"/>
     </row>
-    <row r="252" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="252" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A252" s="2" t="s">
         <v>367</v>
       </c>
@@ -10157,7 +10155,7 @@
       <c r="J252" s="19"/>
       <c r="K252" s="19"/>
     </row>
-    <row r="253" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="253" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A253" s="2" t="s">
         <v>371</v>
       </c>
@@ -10185,7 +10183,7 @@
       <c r="J253" s="19"/>
       <c r="K253" s="19"/>
     </row>
-    <row r="254" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="254" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A254" s="2" t="s">
         <v>816</v>
       </c>
@@ -10223,12 +10221,21 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement/>
 </p:properties>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100AF0C36E9CBDE43468AAB846756A8BA94" ma:contentTypeVersion="0" ma:contentTypeDescription="Crear nuevo documento." ma:contentTypeScope="" ma:versionID="93c275e25462616b2c1de9b58ec156dd">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="3f6edc329ff236629c56e3b879b320d0">
     <xsd:element name="properties">
@@ -10342,16 +10349,15 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DDD49F8-6691-4324-BC0D-0B1E4890A2C6}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{87FEFD23-736F-4CE9-81DA-D9D145B9B572}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
@@ -10366,7 +10372,7 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{A01C7383-C303-4DC2-9970-99C89A193825}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -10380,12 +10386,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3DDD49F8-6691-4324-BC0D-0B1E4890A2C6}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>